<commit_message>
metadata + signature + update struct 514af899c17b300f423af6d75f7413d5d1fbc60b
</commit_message>
<xml_diff>
--- a/spec-tech/ig/StructureDefinition-pdlgc-archive-patient.xlsx
+++ b/spec-tech/ig/StructureDefinition-pdlgc-archive-patient.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="483" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="641" uniqueCount="132">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-16T11:12:17+00:00</t>
+    <t>2026-07-16T21:31:30+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -279,21 +279,21 @@
     <t>Informations éditoriales</t>
   </si>
   <si>
-    <t>pdlgc-archive-patient.IHEXDM</t>
+    <t>pdlgc-archive-patient.PDF</t>
   </si>
   <si>
     <t xml:space="preserve">BackboneElement
 </t>
   </si>
   <si>
-    <t>répertoire IHE_XDM contenant le lot de soumissions des données d'un patient. Nom du répertoire fixé à IHE_XDM</t>
+    <t>Répertoire contenant une copie PDF de tous les documents transportés dans le répertoire IHE_XDM.</t>
   </si>
   <si>
     <t xml:space="preserve">ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
 </t>
   </si>
   <si>
-    <t>pdlgc-archive-patient.IHEXDM.id</t>
+    <t>pdlgc-archive-patient.PDF.id</t>
   </si>
   <si>
     <t xml:space="preserve">string
@@ -309,7 +309,7 @@
     <t>Element.id</t>
   </si>
   <si>
-    <t>pdlgc-archive-patient.IHEXDM.extension</t>
+    <t>pdlgc-archive-patient.PDF.extension</t>
   </si>
   <si>
     <t>extensions
@@ -346,7 +346,7 @@
 ext-1:Must have either extensions or value[x], not both {extension.exists() != value.exists()}</t>
   </si>
   <si>
-    <t>pdlgc-archive-patient.IHEXDM.modifierExtension</t>
+    <t>pdlgc-archive-patient.PDF.modifierExtension</t>
   </si>
   <si>
     <t>extensions
@@ -369,6 +369,31 @@
     <t>BackboneElement.modifierExtension</t>
   </si>
   <si>
+    <t>pdlgc-archive-patient.PDF.documentsPDF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/mos/StructureDefinition/Document
+</t>
+  </si>
+  <si>
+    <t>Documents PDF destinés à la consultation. Ces documents ne sont pas intégrés par le destinataire si le destinataire est une système</t>
+  </si>
+  <si>
+    <t>pdlgc-archive-patient.IHEXDM</t>
+  </si>
+  <si>
+    <t>répertoire IHE_XDM contenant le lot de soumissions des données d'un patient. Nom du répertoire fixé à IHE_XDM</t>
+  </si>
+  <si>
+    <t>pdlgc-archive-patient.IHEXDM.id</t>
+  </si>
+  <si>
+    <t>pdlgc-archive-patient.IHEXDM.extension</t>
+  </si>
+  <si>
+    <t>pdlgc-archive-patient.IHEXDM.modifierExtension</t>
+  </si>
+  <si>
     <t>pdlgc-archive-patient.IHEXDM.SUBSET01</t>
   </si>
   <si>
@@ -395,10 +420,6 @@
   </si>
   <si>
     <t>pdlgc-archive-patient.IHEXDM.SUBSET01.documents</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/mos/StructureDefinition/Document
-</t>
   </si>
   <si>
     <t>Documents de santé du patient</t>
@@ -703,7 +724,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AJ14"/>
+  <dimension ref="A1:AJ19"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="47.92578125" customWidth="true" bestFit="true"/>
@@ -1577,7 +1598,7 @@
         <v>81</v>
       </c>
       <c r="G9" t="s" s="2">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="H9" t="s" s="2">
         <v>73</v>
@@ -1589,13 +1610,13 @@
         <v>73</v>
       </c>
       <c r="K9" t="s" s="2">
-        <v>88</v>
+        <v>115</v>
       </c>
       <c r="L9" t="s" s="2">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="M9" t="s" s="2">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="N9" s="2"/>
       <c r="O9" s="2"/>
@@ -1652,21 +1673,21 @@
         <v>81</v>
       </c>
       <c r="AH9" t="s" s="2">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="AI9" t="s" s="2">
         <v>73</v>
       </c>
       <c r="AJ9" t="s" s="2">
-        <v>90</v>
+        <v>73</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="2">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B10" t="s" s="2">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" t="s" s="2">
@@ -1674,7 +1695,7 @@
       </c>
       <c r="E10" s="2"/>
       <c r="F10" t="s" s="2">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="G10" t="s" s="2">
         <v>81</v>
@@ -1689,13 +1710,13 @@
         <v>73</v>
       </c>
       <c r="K10" t="s" s="2">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="L10" t="s" s="2">
-        <v>93</v>
+        <v>118</v>
       </c>
       <c r="M10" t="s" s="2">
-        <v>94</v>
+        <v>118</v>
       </c>
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>
@@ -1746,10 +1767,10 @@
         <v>73</v>
       </c>
       <c r="AF10" t="s" s="2">
-        <v>95</v>
+        <v>117</v>
       </c>
       <c r="AG10" t="s" s="2">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="AH10" t="s" s="2">
         <v>81</v>
@@ -1758,26 +1779,26 @@
         <v>73</v>
       </c>
       <c r="AJ10" t="s" s="2">
-        <v>73</v>
+        <v>90</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="2">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B11" t="s" s="2">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" t="s" s="2">
-        <v>97</v>
+        <v>73</v>
       </c>
       <c r="E11" s="2"/>
       <c r="F11" t="s" s="2">
         <v>74</v>
       </c>
       <c r="G11" t="s" s="2">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="H11" t="s" s="2">
         <v>73</v>
@@ -1789,17 +1810,15 @@
         <v>73</v>
       </c>
       <c r="K11" t="s" s="2">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="L11" t="s" s="2">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="M11" t="s" s="2">
-        <v>100</v>
-      </c>
-      <c r="N11" t="s" s="2">
-        <v>101</v>
-      </c>
+        <v>94</v>
+      </c>
+      <c r="N11" s="2"/>
       <c r="O11" s="2"/>
       <c r="P11" t="s" s="2">
         <v>73</v>
@@ -1836,43 +1855,43 @@
         <v>73</v>
       </c>
       <c r="AB11" t="s" s="2">
-        <v>102</v>
+        <v>73</v>
       </c>
       <c r="AC11" t="s" s="2">
-        <v>103</v>
+        <v>73</v>
       </c>
       <c r="AD11" t="s" s="2">
         <v>73</v>
       </c>
       <c r="AE11" t="s" s="2">
-        <v>104</v>
+        <v>73</v>
       </c>
       <c r="AF11" t="s" s="2">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="AG11" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AH11" t="s" s="2">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="AI11" t="s" s="2">
         <v>73</v>
       </c>
       <c r="AJ11" t="s" s="2">
-        <v>106</v>
+        <v>73</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="2">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B12" t="s" s="2">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" t="s" s="2">
-        <v>108</v>
+        <v>97</v>
       </c>
       <c r="E12" s="2"/>
       <c r="F12" t="s" s="2">
@@ -1885,26 +1904,24 @@
         <v>73</v>
       </c>
       <c r="I12" t="s" s="2">
-        <v>109</v>
+        <v>73</v>
       </c>
       <c r="J12" t="s" s="2">
-        <v>109</v>
+        <v>73</v>
       </c>
       <c r="K12" t="s" s="2">
         <v>98</v>
       </c>
       <c r="L12" t="s" s="2">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="M12" t="s" s="2">
-        <v>111</v>
+        <v>100</v>
       </c>
       <c r="N12" t="s" s="2">
         <v>101</v>
       </c>
-      <c r="O12" t="s" s="2">
-        <v>112</v>
-      </c>
+      <c r="O12" s="2"/>
       <c r="P12" t="s" s="2">
         <v>73</v>
       </c>
@@ -1940,19 +1957,19 @@
         <v>73</v>
       </c>
       <c r="AB12" t="s" s="2">
-        <v>73</v>
+        <v>102</v>
       </c>
       <c r="AC12" t="s" s="2">
-        <v>73</v>
+        <v>103</v>
       </c>
       <c r="AD12" t="s" s="2">
         <v>73</v>
       </c>
       <c r="AE12" t="s" s="2">
-        <v>73</v>
+        <v>104</v>
       </c>
       <c r="AF12" t="s" s="2">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="AG12" t="s" s="2">
         <v>74</v>
@@ -1969,42 +1986,46 @@
     </row>
     <row r="13">
       <c r="A13" t="s" s="2">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" t="s" s="2">
-        <v>73</v>
+        <v>108</v>
       </c>
       <c r="E13" s="2"/>
       <c r="F13" t="s" s="2">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="G13" t="s" s="2">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="H13" t="s" s="2">
         <v>73</v>
       </c>
       <c r="I13" t="s" s="2">
-        <v>73</v>
+        <v>109</v>
       </c>
       <c r="J13" t="s" s="2">
-        <v>73</v>
+        <v>109</v>
       </c>
       <c r="K13" t="s" s="2">
-        <v>120</v>
+        <v>98</v>
       </c>
       <c r="L13" t="s" s="2">
-        <v>121</v>
+        <v>110</v>
       </c>
       <c r="M13" t="s" s="2">
-        <v>121</v>
-      </c>
-      <c r="N13" s="2"/>
-      <c r="O13" s="2"/>
+        <v>111</v>
+      </c>
+      <c r="N13" t="s" s="2">
+        <v>101</v>
+      </c>
+      <c r="O13" t="s" s="2">
+        <v>112</v>
+      </c>
       <c r="P13" t="s" s="2">
         <v>73</v>
       </c>
@@ -2052,19 +2073,19 @@
         <v>73</v>
       </c>
       <c r="AF13" t="s" s="2">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="AG13" t="s" s="2">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="AH13" t="s" s="2">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="AI13" t="s" s="2">
         <v>73</v>
       </c>
       <c r="AJ13" t="s" s="2">
-        <v>73</v>
+        <v>106</v>
       </c>
     </row>
     <row r="14">
@@ -2083,7 +2104,7 @@
         <v>81</v>
       </c>
       <c r="G14" t="s" s="2">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="H14" t="s" s="2">
         <v>73</v>
@@ -2095,13 +2116,13 @@
         <v>73</v>
       </c>
       <c r="K14" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="L14" t="s" s="2">
         <v>123</v>
       </c>
-      <c r="L14" t="s" s="2">
-        <v>124</v>
-      </c>
       <c r="M14" t="s" s="2">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="N14" s="2"/>
       <c r="O14" s="2"/>
@@ -2158,12 +2179,518 @@
         <v>81</v>
       </c>
       <c r="AH14" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AI14" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AJ14" t="s" s="2">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s" s="2">
+        <v>124</v>
+      </c>
+      <c r="B15" t="s" s="2">
+        <v>124</v>
+      </c>
+      <c r="C15" s="2"/>
+      <c r="D15" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="E15" s="2"/>
+      <c r="F15" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="G15" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="H15" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="I15" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="J15" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="K15" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="L15" t="s" s="2">
+        <v>93</v>
+      </c>
+      <c r="M15" t="s" s="2">
+        <v>94</v>
+      </c>
+      <c r="N15" s="2"/>
+      <c r="O15" s="2"/>
+      <c r="P15" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Q15" s="2"/>
+      <c r="R15" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="S15" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="T15" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="U15" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="V15" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="W15" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="X15" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Y15" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Z15" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AA15" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AB15" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AC15" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AD15" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AE15" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AF15" t="s" s="2">
+        <v>95</v>
+      </c>
+      <c r="AG15" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AH15" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AI15" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AJ15" t="s" s="2">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s" s="2">
+        <v>125</v>
+      </c>
+      <c r="B16" t="s" s="2">
+        <v>125</v>
+      </c>
+      <c r="C16" s="2"/>
+      <c r="D16" t="s" s="2">
+        <v>97</v>
+      </c>
+      <c r="E16" s="2"/>
+      <c r="F16" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="G16" t="s" s="2">
         <v>75</v>
       </c>
-      <c r="AI14" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="AJ14" t="s" s="2">
+      <c r="H16" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="I16" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="J16" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="K16" t="s" s="2">
+        <v>98</v>
+      </c>
+      <c r="L16" t="s" s="2">
+        <v>99</v>
+      </c>
+      <c r="M16" t="s" s="2">
+        <v>100</v>
+      </c>
+      <c r="N16" t="s" s="2">
+        <v>101</v>
+      </c>
+      <c r="O16" s="2"/>
+      <c r="P16" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Q16" s="2"/>
+      <c r="R16" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="S16" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="T16" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="U16" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="V16" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="W16" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="X16" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Y16" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Z16" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AA16" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AB16" t="s" s="2">
+        <v>102</v>
+      </c>
+      <c r="AC16" t="s" s="2">
+        <v>103</v>
+      </c>
+      <c r="AD16" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AE16" t="s" s="2">
+        <v>104</v>
+      </c>
+      <c r="AF16" t="s" s="2">
+        <v>105</v>
+      </c>
+      <c r="AG16" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AH16" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AI16" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AJ16" t="s" s="2">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s" s="2">
+        <v>126</v>
+      </c>
+      <c r="B17" t="s" s="2">
+        <v>126</v>
+      </c>
+      <c r="C17" s="2"/>
+      <c r="D17" t="s" s="2">
+        <v>108</v>
+      </c>
+      <c r="E17" s="2"/>
+      <c r="F17" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="G17" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="H17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="I17" t="s" s="2">
+        <v>109</v>
+      </c>
+      <c r="J17" t="s" s="2">
+        <v>109</v>
+      </c>
+      <c r="K17" t="s" s="2">
+        <v>98</v>
+      </c>
+      <c r="L17" t="s" s="2">
+        <v>110</v>
+      </c>
+      <c r="M17" t="s" s="2">
+        <v>111</v>
+      </c>
+      <c r="N17" t="s" s="2">
+        <v>101</v>
+      </c>
+      <c r="O17" t="s" s="2">
+        <v>112</v>
+      </c>
+      <c r="P17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Q17" s="2"/>
+      <c r="R17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="S17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="T17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="U17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="V17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="W17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="X17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Y17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Z17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AA17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AB17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AC17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AD17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AE17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AF17" t="s" s="2">
+        <v>113</v>
+      </c>
+      <c r="AG17" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AH17" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AI17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AJ17" t="s" s="2">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s" s="2">
+        <v>127</v>
+      </c>
+      <c r="B18" t="s" s="2">
+        <v>127</v>
+      </c>
+      <c r="C18" s="2"/>
+      <c r="D18" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="E18" s="2"/>
+      <c r="F18" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="G18" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="H18" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="I18" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="J18" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="K18" t="s" s="2">
+        <v>128</v>
+      </c>
+      <c r="L18" t="s" s="2">
+        <v>129</v>
+      </c>
+      <c r="M18" t="s" s="2">
+        <v>129</v>
+      </c>
+      <c r="N18" s="2"/>
+      <c r="O18" s="2"/>
+      <c r="P18" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Q18" s="2"/>
+      <c r="R18" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="S18" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="T18" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="U18" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="V18" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="W18" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="X18" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Y18" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Z18" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AA18" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AB18" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AC18" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AD18" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AE18" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AF18" t="s" s="2">
+        <v>127</v>
+      </c>
+      <c r="AG18" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AH18" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AI18" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AJ18" t="s" s="2">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s" s="2">
+        <v>130</v>
+      </c>
+      <c r="B19" t="s" s="2">
+        <v>130</v>
+      </c>
+      <c r="C19" s="2"/>
+      <c r="D19" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="E19" s="2"/>
+      <c r="F19" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="G19" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="H19" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="I19" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="J19" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="K19" t="s" s="2">
+        <v>115</v>
+      </c>
+      <c r="L19" t="s" s="2">
+        <v>131</v>
+      </c>
+      <c r="M19" t="s" s="2">
+        <v>131</v>
+      </c>
+      <c r="N19" s="2"/>
+      <c r="O19" s="2"/>
+      <c r="P19" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Q19" s="2"/>
+      <c r="R19" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="S19" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="T19" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="U19" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="V19" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="W19" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="X19" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Y19" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Z19" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AA19" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AB19" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AC19" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AD19" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AE19" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AF19" t="s" s="2">
+        <v>130</v>
+      </c>
+      <c r="AG19" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AH19" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AI19" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AJ19" t="s" s="2">
         <v>73</v>
       </c>
     </row>

</xml_diff>

<commit_message>
suppression tb concepts + update modèles logiques 2e934d8253f8c7147feaf5abdee23ecf8f59ecc7
</commit_message>
<xml_diff>
--- a/spec-tech/ig/StructureDefinition-pdlgc-archive-patient.xlsx
+++ b/spec-tech/ig/StructureDefinition-pdlgc-archive-patient.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="641" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="672" uniqueCount="134">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-21T16:53:48+00:00</t>
+    <t>2026-07-22T08:07:11+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -266,7 +266,7 @@
 </t>
   </si>
   <si>
-    <t>Informations éditoriales et instructions d'exploitation de l'archive</t>
+    <t>Informations éditoriales et instructions d'exploitation de l'archive.</t>
   </si>
   <si>
     <t>pdlgc-archive-patient.INDEX</t>
@@ -276,7 +276,7 @@
 </t>
   </si>
   <si>
-    <t>Informations éditoriales</t>
+    <t>Informations éditoriales.</t>
   </si>
   <si>
     <t>pdlgc-archive-patient.PDF</t>
@@ -369,20 +369,20 @@
     <t>BackboneElement.modifierExtension</t>
   </si>
   <si>
-    <t>pdlgc-archive-patient.PDF.documentsPDF</t>
+    <t>pdlgc-archive-patient.PDF.documentPDF</t>
   </si>
   <si>
     <t xml:space="preserve">https://interop.esante.gouv.fr/ig/mos/StructureDefinition/Document
 </t>
   </si>
   <si>
-    <t>Documents PDF destinés à la consultation. Ces documents ne sont pas intégrés par le destinataire si le destinataire est une système</t>
+    <t>Document PDF destiné à la consultation. Ces documents ne sont pas intégrés par le destinataire si le destinataire est une système.</t>
   </si>
   <si>
     <t>pdlgc-archive-patient.IHEXDM</t>
   </si>
   <si>
-    <t>répertoire IHE_XDM contenant le lot de soumissions des données d'un patient. Nom du répertoire fixé à IHE_XDM</t>
+    <t>répertoire IHE_XDM contenant le lot de soumissions des données d'un patient. Nom du répertoire fixé à IHE_XDM.</t>
   </si>
   <si>
     <t>pdlgc-archive-patient.IHEXDM.id</t>
@@ -397,7 +397,7 @@
     <t>pdlgc-archive-patient.IHEXDM.SUBSET01</t>
   </si>
   <si>
-    <t>lot de soumission contenant les données d'un patient</t>
+    <t>lot de soumission contenant les données d'un patient.</t>
   </si>
   <si>
     <t>pdlgc-archive-patient.IHEXDM.SUBSET01.id</t>
@@ -416,13 +416,19 @@
 </t>
   </si>
   <si>
-    <t>métadonnées associées aux documents du lot de soumission</t>
-  </si>
-  <si>
-    <t>pdlgc-archive-patient.IHEXDM.SUBSET01.documents</t>
-  </si>
-  <si>
-    <t>Documents de santé du patient</t>
+    <t>métadonnées du lot de soumission, conforme au profil IHE XDM, décrivant les documents patient qu'il accompagne.</t>
+  </si>
+  <si>
+    <t>pdlgc-archive-patient.IHEXDM.SUBSET01.documentPivot</t>
+  </si>
+  <si>
+    <t>Données structurées du périmètres pivot, concernant les informations administratives et médicales du patient. Leur export est obligatoire.</t>
+  </si>
+  <si>
+    <t>pdlgc-archive-patient.IHEXDM.SUBSET01.documentHorsPivot</t>
+  </si>
+  <si>
+    <t>Données structurées hors périmètre pivot. Leur export est facultatif.</t>
   </si>
 </sst>
 </file>
@@ -724,11 +730,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AJ19"/>
+  <dimension ref="A1:AJ20"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="47.92578125" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="47.92578125" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="49.109375" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="49.109375" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="10.8515625" customWidth="true" bestFit="true" hidden="true"/>
     <col min="4" max="4" width="18.19140625" customWidth="true" bestFit="true" hidden="true"/>
     <col min="5" max="5" width="5.80859375" customWidth="true" bestFit="true"/>
@@ -758,7 +764,7 @@
     <col min="29" max="29" width="36.0390625" customWidth="true" bestFit="true"/>
     <col min="30" max="30" width="14.7578125" customWidth="true" bestFit="true"/>
     <col min="31" max="31" width="12.359375" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="32" max="32" width="42.42578125" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="32" max="32" width="49.109375" customWidth="true" bestFit="true" hidden="true"/>
     <col min="33" max="33" width="9.046875" customWidth="true" bestFit="true" hidden="true"/>
     <col min="34" max="34" width="9.46484375" customWidth="true" bestFit="true"/>
     <col min="35" max="35" width="100.703125" customWidth="true"/>
@@ -2694,6 +2700,106 @@
         <v>73</v>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="s" s="2">
+        <v>132</v>
+      </c>
+      <c r="B20" t="s" s="2">
+        <v>132</v>
+      </c>
+      <c r="C20" s="2"/>
+      <c r="D20" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="E20" s="2"/>
+      <c r="F20" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="G20" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="H20" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="I20" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="J20" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="K20" t="s" s="2">
+        <v>115</v>
+      </c>
+      <c r="L20" t="s" s="2">
+        <v>133</v>
+      </c>
+      <c r="M20" t="s" s="2">
+        <v>133</v>
+      </c>
+      <c r="N20" s="2"/>
+      <c r="O20" s="2"/>
+      <c r="P20" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Q20" s="2"/>
+      <c r="R20" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="S20" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="T20" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="U20" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="V20" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="W20" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="X20" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Y20" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Z20" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AA20" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AB20" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AC20" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AD20" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AE20" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AF20" t="s" s="2">
+        <v>132</v>
+      </c>
+      <c r="AG20" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AH20" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AI20" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AJ20" t="s" s="2">
+        <v>73</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
correctifs QA + hamronisation cs vs + redaction README IG 41ea2840b69f4baaefbf2bccb6bd8c8e58c2e971
</commit_message>
<xml_diff>
--- a/spec-tech/ig/StructureDefinition-pdlgc-archive-patient.xlsx
+++ b/spec-tech/ig/StructureDefinition-pdlgc-archive-patient.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-22T10:39:39+00:00</t>
+    <t>2026-07-22T17:16:50+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -256,7 +256,7 @@
     <t>Base</t>
   </si>
   <si>
-    <t>pdlgc-archive-patient.README</t>
+    <t>pdlgc-archive-patient.readme</t>
   </si>
   <si>
     <t>1</t>
@@ -269,7 +269,7 @@
     <t>Informations éditoriales et instructions d'exploitation de l'archive.</t>
   </si>
   <si>
-    <t>pdlgc-archive-patient.INDEX</t>
+    <t>pdlgc-archive-patient.index</t>
   </si>
   <si>
     <t xml:space="preserve">https://interop.esante.gouv.fr/ig/fhir/pdlgc/StructureDefinition/pdlgc-index
@@ -379,37 +379,37 @@
     <t>Document PDF destiné à la consultation. Ces documents ne sont pas intégrés par le destinataire si le destinataire est une système.</t>
   </si>
   <si>
-    <t>pdlgc-archive-patient.IHEXDM</t>
+    <t>pdlgc-archive-patient.iheXdm</t>
   </si>
   <si>
     <t>répertoire IHE_XDM contenant le lot de soumissions des données d'un patient. Nom du répertoire fixé à IHE_XDM.</t>
   </si>
   <si>
-    <t>pdlgc-archive-patient.IHEXDM.id</t>
-  </si>
-  <si>
-    <t>pdlgc-archive-patient.IHEXDM.extension</t>
-  </si>
-  <si>
-    <t>pdlgc-archive-patient.IHEXDM.modifierExtension</t>
-  </si>
-  <si>
-    <t>pdlgc-archive-patient.IHEXDM.SUBSET01</t>
+    <t>pdlgc-archive-patient.iheXdm.id</t>
+  </si>
+  <si>
+    <t>pdlgc-archive-patient.iheXdm.extension</t>
+  </si>
+  <si>
+    <t>pdlgc-archive-patient.iheXdm.modifierExtension</t>
+  </si>
+  <si>
+    <t>pdlgc-archive-patient.iheXdm.subset01</t>
   </si>
   <si>
     <t>lot de soumission contenant les données d'un patient.</t>
   </si>
   <si>
-    <t>pdlgc-archive-patient.IHEXDM.SUBSET01.id</t>
-  </si>
-  <si>
-    <t>pdlgc-archive-patient.IHEXDM.SUBSET01.extension</t>
-  </si>
-  <si>
-    <t>pdlgc-archive-patient.IHEXDM.SUBSET01.modifierExtension</t>
-  </si>
-  <si>
-    <t>pdlgc-archive-patient.IHEXDM.SUBSET01.METADATA</t>
+    <t>pdlgc-archive-patient.iheXdm.subset01.id</t>
+  </si>
+  <si>
+    <t>pdlgc-archive-patient.iheXdm.subset01.extension</t>
+  </si>
+  <si>
+    <t>pdlgc-archive-patient.iheXdm.subset01.modifierExtension</t>
+  </si>
+  <si>
+    <t>pdlgc-archive-patient.iheXdm.subset01.metadata</t>
   </si>
   <si>
     <t xml:space="preserve">https://interop.esante.gouv.fr/ig/fhir/pdlgc/StructureDefinition/pdlgc-metadata
@@ -419,13 +419,13 @@
     <t>métadonnées du lot de soumission, conforme au profil IHE XDM, décrivant les documents patient qu'il accompagne.</t>
   </si>
   <si>
-    <t>pdlgc-archive-patient.IHEXDM.SUBSET01.documentPivot</t>
+    <t>pdlgc-archive-patient.iheXdm.subset01.documentPivot</t>
   </si>
   <si>
     <t>Données structurées du périmètres pivot, concernant les informations administratives et médicales du patient. Leur export est obligatoire.</t>
   </si>
   <si>
-    <t>pdlgc-archive-patient.IHEXDM.SUBSET01.documentHorsPivot</t>
+    <t>pdlgc-archive-patient.iheXdm.subset01.documentHorsPivot</t>
   </si>
   <si>
     <t>Données structurées hors périmètre pivot. Leur export est facultatif.</t>
@@ -733,8 +733,8 @@
   <dimension ref="A1:AJ20"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="49.109375" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="49.109375" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="47.87109375" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="47.87109375" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="10.8515625" customWidth="true" bestFit="true" hidden="true"/>
     <col min="4" max="4" width="18.19140625" customWidth="true" bestFit="true" hidden="true"/>
     <col min="5" max="5" width="5.80859375" customWidth="true" bestFit="true"/>
@@ -764,7 +764,7 @@
     <col min="29" max="29" width="36.0390625" customWidth="true" bestFit="true"/>
     <col min="30" max="30" width="14.7578125" customWidth="true" bestFit="true"/>
     <col min="31" max="31" width="12.359375" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="32" max="32" width="49.109375" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="32" max="32" width="47.87109375" customWidth="true" bestFit="true" hidden="true"/>
     <col min="33" max="33" width="9.046875" customWidth="true" bestFit="true" hidden="true"/>
     <col min="34" max="34" width="9.46484375" customWidth="true" bestFit="true"/>
     <col min="35" max="35" width="100.703125" customWidth="true"/>

</xml_diff>